<commit_message>
Syncing before I try to fix the data curation
</commit_message>
<xml_diff>
--- a/timeline.xlsx
+++ b/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahm\projects\loc_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793D788B-781F-49EE-A77C-A845B6CAB783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE823A53-CD75-45B4-865D-9EFCF2375C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6B063EC0-67D1-47C9-8561-C8AF2753B48C}"/>
   </bookViews>
@@ -271,7 +271,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -287,6 +287,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -457,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -521,6 +527,21 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1138,22 +1159,22 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B5" s="8">
+      <c r="B5" s="22">
         <v>1</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="20">
+      <c r="E5" s="25">
         <v>37865</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="11"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="26"/>
     </row>
     <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B6" s="8">

</xml_diff>